<commit_message>
Added the leetcode tracker that also has logic for each problem
</commit_message>
<xml_diff>
--- a/LeetCode/NeetCode_Tracker.xlsx
+++ b/LeetCode/NeetCode_Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyPersonalProjects\Python_Journey\LeetCode\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyPersonalProjects\Cpp_Journey\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE247B2-E72A-40A7-8F21-1F3A173F32AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A778E2-A099-4756-A7A7-07BC79A598B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{7A33F154-936F-4041-96A3-17E59C2ECE87}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="94">
   <si>
     <t>Status</t>
   </si>
@@ -296,6 +296,16 @@
   </si>
   <si>
     <t>LOGIC TRICK</t>
+  </si>
+  <si>
+    <t>HashMap(value, index). 
+Need = Target - value 
+If can find return else add entry to HashMap</t>
+  </si>
+  <si>
+    <t>Use Set
+Add all elements
+Compare Size of set and array</t>
   </si>
 </sst>
 </file>
@@ -826,16 +836,27 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1197,7 +1218,7 @@
     <col min="1" max="1" width="28.265625" customWidth="1"/>
     <col min="2" max="2" width="54" customWidth="1"/>
     <col min="3" max="3" width="9.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="54.53125" customWidth="1"/>
+    <col min="4" max="4" width="37.33203125" customWidth="1"/>
     <col min="9" max="9" width="9.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1215,842 +1236,917 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+    <row r="2" spans="1:9" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>1</v>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="A3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="C3" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="8"/>
+    </row>
+    <row r="4" spans="1:9" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>1</v>
+      <c r="C4" s="4"/>
+      <c r="D4" s="10" t="s">
+        <v>93</v>
       </c>
       <c r="H4" s="4"/>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="7" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="A5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C5" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="8"/>
       <c r="H5" s="5"/>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+      <c r="A6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C6" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="8"/>
       <c r="H6" s="3"/>
       <c r="I6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+      <c r="A7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C7" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" s="8"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+      <c r="A8" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C8" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="8"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+      <c r="A9" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C9" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="8"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+      <c r="A10" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C10" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+      <c r="A11" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C11" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="8"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
+      <c r="A12" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C12" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="8"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
+      <c r="A13" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C13" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D13" s="8"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
+      <c r="A14" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C14" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="8"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
+      <c r="A15" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C15" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15" s="8"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
+      <c r="A16" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
+      <c r="C16" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" s="8"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
+      <c r="C17" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" s="8"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A18" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
+      <c r="C18" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="8"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A19" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
+      <c r="C19" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D19" s="8"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
+      <c r="C20" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20" s="8"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
+      <c r="C21" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" s="8"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A22" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
+      <c r="C22" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D22" s="8"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A23" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
+      <c r="C23" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D23" s="8"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A24" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
+      <c r="C24" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D24" s="8"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A25" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
+      <c r="C25" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25" s="8"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A26" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
+      <c r="C26" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" s="8"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A27" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
+      <c r="C27" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="8"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A28" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
+      <c r="C28" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D28" s="8"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A29" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
+      <c r="C29" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29" s="8"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A30" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
+      <c r="C30" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D30" s="8"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A31" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
+      <c r="C31" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31" s="8"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A32" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C32" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
+      <c r="C32" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32" s="8"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A33" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C33" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
+      <c r="C33" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" s="8"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A34" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C34" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
+      <c r="C34" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D34" s="8"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A35" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C35" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
+      <c r="C35" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D35" s="8"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A36" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
+      <c r="C36" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D36" s="8"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A37" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
+      <c r="C37" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37" s="8"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A38" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
+      <c r="C38" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D38" s="8"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A39" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C39" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
+      <c r="C39" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D39" s="8"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A40" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C40" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
+      <c r="C40" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D40" s="8"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A41" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C41" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
+      <c r="C41" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D41" s="8"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A42" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C42" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A43" t="s">
+      <c r="C42" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D42" s="8"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A43" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C43" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A44" t="s">
+      <c r="C43" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D43" s="8"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A44" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C44" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A45" t="s">
+      <c r="C44" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D44" s="8"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A45" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C45" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A46" t="s">
+      <c r="C45" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D45" s="8"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A46" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C46" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A47" t="s">
+      <c r="C46" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D46" s="8"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A47" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C47" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
+      <c r="C47" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D47" s="8"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A48" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C48" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A49" t="s">
+      <c r="C48" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D48" s="8"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A49" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C49" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A50" t="s">
+      <c r="C49" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D49" s="8"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A50" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C50" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
+      <c r="C50" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D50" s="8"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A51" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C51" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
+      <c r="C51" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D51" s="8"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A52" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C52" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A53" t="s">
+      <c r="C52" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D52" s="8"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A53" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C53" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A54" t="s">
+      <c r="C53" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D53" s="8"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A54" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C54" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
+      <c r="C54" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D54" s="8"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A55" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C55" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A56" t="s">
+      <c r="C55" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D55" s="8"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A56" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="C56" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A57" t="s">
+      <c r="C56" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D56" s="8"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A57" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C57" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A58" t="s">
+      <c r="C57" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D57" s="8"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A58" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C58" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A59" t="s">
+      <c r="C58" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D58" s="8"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A59" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C59" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A60" t="s">
+      <c r="C59" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D59" s="8"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A60" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C60" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A61" t="s">
+      <c r="C60" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D60" s="8"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A61" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C61" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A62" t="s">
+      <c r="C61" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D61" s="8"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A62" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C62" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A63" t="s">
+      <c r="C62" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D62" s="8"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A63" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C63" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A64" t="s">
+      <c r="C63" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D63" s="8"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A64" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="C64" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A65" t="s">
+      <c r="C64" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D64" s="8"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A65" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="C65" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A66" t="s">
+      <c r="C65" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D65" s="8"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A66" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C66" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A67" t="s">
+      <c r="C66" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D66" s="8"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A67" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C67" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A68" t="s">
+      <c r="C67" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D67" s="8"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A68" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="C68" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A69" t="s">
+      <c r="C68" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D68" s="8"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A69" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C69" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A70" t="s">
+      <c r="C69" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D69" s="8"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A70" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C70" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A71" t="s">
+      <c r="C70" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D70" s="8"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A71" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="C71" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A72" t="s">
+      <c r="C71" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D71" s="8"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A72" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C72" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A73" t="s">
+      <c r="C72" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D72" s="8"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A73" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C73" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A74" t="s">
+      <c r="C73" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D73" s="8"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A74" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C74" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A75" t="s">
+      <c r="C74" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D74" s="8"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A75" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="C75" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A76" t="s">
+      <c r="C75" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D75" s="8"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A76" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C76" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="C76" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D76" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>